<commit_message>
update code journal details and shared month export and file upload
</commit_message>
<xml_diff>
--- a/CBS.FrontDesk.UI/AppFiles/ShareMonthUpload/Anual data.xlsx
+++ b/CBS.FrontDesk.UI/AppFiles/ShareMonthUpload/Anual data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9C2B866B-475F-46DB-8C55-3B69CCE98ADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{765477ED-A3BE-4291-9660-EFFE2BD77DC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{1815F049-E94B-4D50-AE2F-565BEF23DC67}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{1815F049-E94B-4D50-AE2F-565BEF23DC67}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,17 +25,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
-  <si>
-    <t>BAPCCUL</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">Branch Name : </t>
   </si>
   <si>
-    <t>Biyem-Assi</t>
-  </si>
-  <si>
     <t xml:space="preserve">Branch Code : </t>
   </si>
   <si>
@@ -97,13 +91,25 @@
   </si>
   <si>
     <t xml:space="preserve"> Anual Shared Month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Affiliate </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Branch name </t>
+  </si>
+  <si>
+    <t>branch code</t>
+  </si>
+  <si>
+    <t>Principal Amount</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,13 +128,6 @@
     <font>
       <sz val="16"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="5" tint="-0.249977111117893"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -154,7 +153,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -211,36 +210,77 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -555,213 +595,255 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A4242A-5EDC-4AEE-9F62-510D2F80FE32}">
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.6640625" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="42.5546875" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
+      <c r="A1" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="18"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="B2" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="9"/>
+      <c r="D2" s="10"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B3" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="9"/>
+      <c r="D3" s="10"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4"/>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="B4" s="11">
+        <v>46022</v>
+      </c>
+      <c r="C4" s="9"/>
+      <c r="D4" s="10"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B5" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="9"/>
+      <c r="D5" s="10"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9">
+        <v>10</v>
+      </c>
+      <c r="C6" s="9"/>
+      <c r="D6" s="10"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="10"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="16"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>1</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="13">
+        <v>10000</v>
+      </c>
+      <c r="D10" s="10">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>2</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="13">
+        <v>15000</v>
+      </c>
+      <c r="D11" s="10">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
         <v>3</v>
       </c>
-      <c r="C3" s="4"/>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="B12" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="13">
+        <v>4000</v>
+      </c>
+      <c r="D12" s="10">
+        <v>560000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
         <v>4</v>
       </c>
-      <c r="B4" s="5">
-        <v>46022</v>
-      </c>
-      <c r="C4" s="4"/>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="B13" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="13">
+        <v>5000</v>
+      </c>
+      <c r="D13" s="10">
+        <v>740000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
         <v>5</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B14" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="13">
+        <v>600000</v>
+      </c>
+      <c r="D14" s="10">
+        <v>78000</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
         <v>6</v>
       </c>
-      <c r="C5" s="4"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+      <c r="B15" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="13">
+        <v>450000</v>
+      </c>
+      <c r="D15" s="10">
+        <v>67000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
         <v>7</v>
       </c>
-      <c r="B6" s="4">
-        <v>1000</v>
-      </c>
-      <c r="C6" s="4"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
+      <c r="B16" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="13">
+        <v>90000</v>
+      </c>
+      <c r="D16" s="10">
+        <v>890000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
         <v>8</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B17" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="13">
+        <v>670000</v>
+      </c>
+      <c r="D17" s="10">
+        <v>900000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
         <v>9</v>
       </c>
-      <c r="C7" s="4"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
+      <c r="B18" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="13">
+        <v>34000</v>
+      </c>
+      <c r="D18" s="10">
+        <v>43000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="4">
         <v>10</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="10">
-        <v>1</v>
-      </c>
-      <c r="B10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10">
-        <v>10000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="10">
-        <v>2</v>
-      </c>
-      <c r="B11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11">
-        <v>15000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="10">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12">
-        <v>4000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="10">
-        <v>4</v>
-      </c>
-      <c r="B13" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="10">
-        <v>5</v>
-      </c>
-      <c r="B14" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14">
-        <v>600000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="10">
-        <v>6</v>
-      </c>
-      <c r="B15" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15">
-        <v>450000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="10">
-        <v>7</v>
-      </c>
-      <c r="B16" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16">
-        <v>90000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="10">
-        <v>8</v>
-      </c>
-      <c r="B17" t="s">
+      <c r="B19" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C17">
-        <v>670000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="10">
-        <v>9</v>
-      </c>
-      <c r="B18" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18">
-        <v>34000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="11">
-        <v>10</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" s="12">
+      <c r="C19" s="5">
         <v>65000</v>
+      </c>
+      <c r="D19" s="14">
+        <v>23000</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A8:D8"/>
+    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update on share month , end of year , journal ex
</commit_message>
<xml_diff>
--- a/CBS.FrontDesk.UI/AppFiles/ShareMonthUpload/Anual data.xlsx
+++ b/CBS.FrontDesk.UI/AppFiles/ShareMonthUpload/Anual data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{765477ED-A3BE-4291-9660-EFFE2BD77DC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBDA10EA-CBC3-4D6D-896A-4C2FA73E7430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{1815F049-E94B-4D50-AE2F-565BEF23DC67}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t xml:space="preserve">Branch Name : </t>
   </si>
@@ -100,9 +100,6 @@
   </si>
   <si>
     <t>branch code</t>
-  </si>
-  <si>
-    <t>Principal Amount</t>
   </si>
 </sst>
 </file>
@@ -153,7 +150,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -210,76 +207,35 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -595,232 +551,193 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A4242A-5EDC-4AEE-9F62-510D2F80FE32}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36.6640625" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="42.5546875" customWidth="1"/>
-    <col min="4" max="4" width="21.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="21" x14ac:dyDescent="0.4">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.4">
+      <c r="A1" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="18"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="10"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C2" s="11"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="10"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C3" s="11"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="12">
         <v>46022</v>
       </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="10"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C4" s="11"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="9"/>
-      <c r="D5" s="10"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C5" s="11"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="11">
         <v>10</v>
       </c>
-      <c r="C6" s="9"/>
-      <c r="D6" s="10"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C6" s="11"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="9"/>
-      <c r="D7" s="10"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
+      <c r="C7" s="11"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
-      <c r="D8" s="16"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B8" s="8"/>
+      <c r="C8" s="8"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="B9" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>1</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10">
         <v>10000</v>
       </c>
-      <c r="D10" s="10">
-        <v>5000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>2</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11">
         <v>15000</v>
       </c>
-      <c r="D11" s="10">
-        <v>30000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>3</v>
       </c>
-      <c r="B12" s="13" t="s">
+      <c r="B12" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12">
         <v>4000</v>
       </c>
-      <c r="D12" s="10">
-        <v>560000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>4</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="B13" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13">
         <v>5000</v>
       </c>
-      <c r="D13" s="10">
-        <v>740000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>5</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14">
         <v>600000</v>
       </c>
-      <c r="D14" s="10">
-        <v>78000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>6</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" t="s">
         <v>16</v>
       </c>
-      <c r="C15" s="13">
+      <c r="C15">
         <v>450000</v>
       </c>
-      <c r="D15" s="10">
-        <v>67000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>7</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="13">
+      <c r="C16">
         <v>90000</v>
       </c>
-      <c r="D16" s="10">
-        <v>890000</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>8</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" t="s">
         <v>18</v>
       </c>
-      <c r="C17" s="13">
+      <c r="C17">
         <v>670000</v>
       </c>
-      <c r="D17" s="10">
-        <v>900000</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>9</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C18">
         <v>34000</v>
       </c>
-      <c r="D18" s="10">
-        <v>43000</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>10</v>
       </c>
@@ -830,20 +747,17 @@
       <c r="C19" s="5">
         <v>65000</v>
       </c>
-      <c r="D19" s="14">
-        <v>23000</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A8:D8"/>
-    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>